<commit_message>
Update data files, scripts, and notebook
Modified binary data files (Data/Clean/base_indices.dta, tabla_indices.xlsx, tabla_indices_mapas.xlsx) and updated document Guion_Audiovisual_Mediterraneos_v2.docx. Enhanced Scripts/09_Construccion_Indices.do with simple summary loops and tabulations for diagnostics. Updated Scripts/10_script_generacion_graficos.ipynb: fixed local paths to user 'anton', added a pip install hint, normalized execution counts/outputs, added a new IDL (Indice de Digitalizacion Local) summary block (general, by hot_zone, and gap calculation), and adjusted notebook metadata. Removed temporary swap file Scripts/~08_Construccion_Base_Datos..do.stswp.
</commit_message>
<xml_diff>
--- a/Data/Clean/tabla_indices.xlsx
+++ b/Data/Clean/tabla_indices.xlsx
@@ -1,26 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
-  <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jessi\OneDrive\Documents\GitHub\DoingEconomics_Proyect\Data\Clean\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB03F755-3554-4EF4-809C-12224E82FBFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Indices" sheetId="1" r:id="rId1"/>
+    <sheet name="Indices" sheetId="1" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="125725" fullCalcOnLoad="true"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1386" uniqueCount="306">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="1386" uniqueCount="306">
   <si>
     <t>Restaurante con encuesta aplicada (1=Si, 0=No)</t>
   </si>
@@ -943,11 +936,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
-    <numFmt numFmtId="169" formatCode="0.0000000"/>
-  </numFmts>
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <fonts count="1">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -969,363 +959,27 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
+    <border/>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="true"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
-  <a:themeElements>
-    <a:clrScheme name="Office">
-      <a:dk1>
-        <a:sysClr val="windowText" lastClr="000000"/>
-      </a:dk1>
-      <a:lt1>
-        <a:sysClr val="window" lastClr="FFFFFF"/>
-      </a:lt1>
-      <a:dk2>
-        <a:srgbClr val="0E2841"/>
-      </a:dk2>
-      <a:lt2>
-        <a:srgbClr val="E8E8E8"/>
-      </a:lt2>
-      <a:accent1>
-        <a:srgbClr val="156082"/>
-      </a:accent1>
-      <a:accent2>
-        <a:srgbClr val="E97132"/>
-      </a:accent2>
-      <a:accent3>
-        <a:srgbClr val="196B24"/>
-      </a:accent3>
-      <a:accent4>
-        <a:srgbClr val="0F9ED5"/>
-      </a:accent4>
-      <a:accent5>
-        <a:srgbClr val="A02B93"/>
-      </a:accent5>
-      <a:accent6>
-        <a:srgbClr val="4EA72E"/>
-      </a:accent6>
-      <a:hlink>
-        <a:srgbClr val="467886"/>
-      </a:hlink>
-      <a:folHlink>
-        <a:srgbClr val="96607D"/>
-      </a:folHlink>
-    </a:clrScheme>
-    <a:fontScheme name="Office">
-      <a:majorFont>
-        <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック Light"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线 Light"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Times New Roman"/>
-        <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="MoolBoran"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Times New Roman"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
-      </a:majorFont>
-      <a:minorFont>
-        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Arial"/>
-        <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="DaunPenh"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Arial"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
-      </a:minorFont>
-    </a:fontScheme>
-    <a:fmtScheme name="Office">
-      <a:fillStyleLst>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="110000"/>
-                <a:satMod val="105000"/>
-                <a:tint val="67000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="103000"/>
-                <a:tint val="73000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="109000"/>
-                <a:tint val="81000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
-        </a:gradFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:satMod val="103000"/>
-                <a:lumMod val="102000"/>
-                <a:tint val="94000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:satMod val="110000"/>
-                <a:lumMod val="100000"/>
-                <a:shade val="100000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="99000"/>
-                <a:satMod val="120000"/>
-                <a:shade val="78000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
-        </a:gradFill>
-      </a:fillStyleLst>
-      <a:lnStyleLst>
-        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-      </a:lnStyleLst>
-      <a:effectStyleLst>
-        <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="63000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-        </a:effectStyle>
-      </a:effectStyleLst>
-      <a:bgFillStyleLst>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="phClr">
-            <a:tint val="95000"/>
-            <a:satMod val="170000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="93000"/>
-                <a:satMod val="150000"/>
-                <a:shade val="98000"/>
-                <a:lumMod val="102000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:tint val="98000"/>
-                <a:satMod val="130000"/>
-                <a:shade val="90000"/>
-                <a:lumMod val="103000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="63000"/>
-                <a:satMod val="120000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
-        </a:gradFill>
-      </a:bgFillStyleLst>
-    </a:fmtScheme>
-  </a:themeElements>
-  <a:objectDefaults>
-    <a:lnDef>
-      <a:spPr/>
-      <a:bodyPr/>
-      <a:lstStyle/>
-      <a:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </a:style>
-    </a:lnDef>
-  </a:objectDefaults>
-  <a:extraClrSchemeLst/>
-  <a:extLst>
-    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
-    </a:ext>
-  </a:extLst>
-</a:theme>
-</file>
-
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:CM36"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="73" max="73" width="10.44140625" bestFit="1" customWidth="1"/>
-    <col min="74" max="74" width="12.109375" bestFit="1" customWidth="1"/>
-  </cols>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:91" x14ac:dyDescent="0.3">
+    <row r="1">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1600,7 +1254,7 @@
         <v>305</v>
       </c>
     </row>
-    <row r="2" spans="1:91" x14ac:dyDescent="0.3">
+    <row r="2">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -1710,7 +1364,7 @@
         <v>10053</v>
       </c>
       <c r="AK2" s="1">
-        <v>4.7</v>
+        <v>4.7000000000000002</v>
       </c>
       <c r="AL2" s="1">
         <v>1</v>
@@ -1719,7 +1373,7 @@
         <v>190</v>
       </c>
       <c r="AN2" s="1">
-        <v>3.7</v>
+        <v>3.7000000000000002</v>
       </c>
       <c r="AO2" t="s">
         <v>163</v>
@@ -1817,10 +1471,10 @@
       <c r="BT2" s="1">
         <v>0</v>
       </c>
-      <c r="BU2" s="2">
+      <c r="BU2" s="1">
         <v>4.6676060000000001</v>
       </c>
-      <c r="BV2" s="2">
+      <c r="BV2" s="1">
         <v>-74.054133999999991</v>
       </c>
       <c r="BW2" t="s">
@@ -1875,7 +1529,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:91" x14ac:dyDescent="0.3">
+    <row r="3">
       <c r="A3" s="1">
         <v>1</v>
       </c>
@@ -1985,7 +1639,7 @@
         <v>7987</v>
       </c>
       <c r="AK3" s="1">
-        <v>4.7</v>
+        <v>4.7000000000000002</v>
       </c>
       <c r="AL3" s="1">
         <v>1</v>
@@ -2092,10 +1746,10 @@
       <c r="BT3" s="1">
         <v>0</v>
       </c>
-      <c r="BU3" s="2">
+      <c r="BU3" s="1">
         <v>4.6672186999999994</v>
       </c>
-      <c r="BV3" s="2">
+      <c r="BV3" s="1">
         <v>-74.054656800000004</v>
       </c>
       <c r="BW3" t="s">
@@ -2150,7 +1804,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:91" x14ac:dyDescent="0.3">
+    <row r="4">
       <c r="A4" s="1">
         <v>1</v>
       </c>
@@ -2269,7 +1923,7 @@
         <v>231</v>
       </c>
       <c r="AN4" s="1">
-        <v>3.9</v>
+        <v>3.8999999999999999</v>
       </c>
       <c r="AO4" t="s">
         <v>165</v>
@@ -2367,10 +2021,10 @@
       <c r="BT4" s="1">
         <v>0</v>
       </c>
-      <c r="BU4" s="2">
+      <c r="BU4" s="1">
         <v>4.6143874999999994</v>
       </c>
-      <c r="BV4" s="2">
+      <c r="BV4" s="1">
         <v>-74.066146599999996</v>
       </c>
       <c r="BW4" t="s">
@@ -2425,7 +2079,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:91" x14ac:dyDescent="0.3">
+    <row r="5">
       <c r="A5" s="1">
         <v>1</v>
       </c>
@@ -2544,7 +2198,7 @@
         <v>825</v>
       </c>
       <c r="AN5" s="1">
-        <v>4.3</v>
+        <v>4.2999999999999998</v>
       </c>
       <c r="AO5" t="s">
         <v>166</v>
@@ -2642,10 +2296,10 @@
       <c r="BT5" s="1">
         <v>0</v>
       </c>
-      <c r="BU5" s="2">
+      <c r="BU5" s="1">
         <v>4.6768090999999998</v>
       </c>
-      <c r="BV5" s="2">
+      <c r="BV5" s="1">
         <v>-74.047285700000003</v>
       </c>
       <c r="BW5" t="s">
@@ -2700,7 +2354,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:91" x14ac:dyDescent="0.3">
+    <row r="6">
       <c r="A6" s="1">
         <v>1</v>
       </c>
@@ -2819,7 +2473,7 @@
         <v>529</v>
       </c>
       <c r="AN6" s="1">
-        <v>4.3</v>
+        <v>4.2999999999999998</v>
       </c>
       <c r="AO6" t="s">
         <v>167</v>
@@ -2917,10 +2571,10 @@
       <c r="BT6" s="1">
         <v>0</v>
       </c>
-      <c r="BU6" s="2">
+      <c r="BU6" s="1">
         <v>4.6702380000000003</v>
       </c>
-      <c r="BV6" s="2">
+      <c r="BV6" s="1">
         <v>-74.053262000000004</v>
       </c>
       <c r="BW6" t="s">
@@ -2975,7 +2629,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:91" x14ac:dyDescent="0.3">
+    <row r="7">
       <c r="A7" s="1">
         <v>1</v>
       </c>
@@ -3094,7 +2748,7 @@
         <v>114</v>
       </c>
       <c r="AN7" s="1">
-        <v>3.9</v>
+        <v>3.8999999999999999</v>
       </c>
       <c r="AO7" t="s">
         <v>168</v>
@@ -3192,10 +2846,10 @@
       <c r="BT7" s="1">
         <v>0</v>
       </c>
-      <c r="BU7" s="2">
+      <c r="BU7" s="1">
         <v>4.6690924999999996</v>
       </c>
-      <c r="BV7" s="2">
+      <c r="BV7" s="1">
         <v>-74.053077899999991</v>
       </c>
       <c r="BW7" t="s">
@@ -3250,7 +2904,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:91" x14ac:dyDescent="0.3">
+    <row r="8">
       <c r="A8" s="1">
         <v>1</v>
       </c>
@@ -3369,7 +3023,7 @@
         <v>419</v>
       </c>
       <c r="AN8" s="1">
-        <v>4.3</v>
+        <v>4.2999999999999998</v>
       </c>
       <c r="AO8" t="s">
         <v>169</v>
@@ -3467,10 +3121,10 @@
       <c r="BT8" s="1">
         <v>0</v>
       </c>
-      <c r="BU8" s="2">
+      <c r="BU8" s="1">
         <v>4.6144970000000001</v>
       </c>
-      <c r="BV8" s="2">
+      <c r="BV8" s="1">
         <v>-74.068920199999994</v>
       </c>
       <c r="BW8" t="s">
@@ -3525,7 +3179,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:91" x14ac:dyDescent="0.3">
+    <row r="9">
       <c r="A9" s="1">
         <v>1</v>
       </c>
@@ -3644,7 +3298,7 @@
         <v>16</v>
       </c>
       <c r="AN9" s="1">
-        <v>3.9</v>
+        <v>3.8999999999999999</v>
       </c>
       <c r="AO9" t="s">
         <v>170</v>
@@ -3742,10 +3396,10 @@
       <c r="BT9" s="1">
         <v>0</v>
       </c>
-      <c r="BU9" s="2">
+      <c r="BU9" s="1">
         <v>4.6963597000000004</v>
       </c>
-      <c r="BV9" s="2">
+      <c r="BV9" s="1">
         <v>-74.030839300000011</v>
       </c>
       <c r="BW9" t="s">
@@ -3800,7 +3454,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:91" x14ac:dyDescent="0.3">
+    <row r="10">
       <c r="A10" s="1">
         <v>1</v>
       </c>
@@ -4017,10 +3671,10 @@
       <c r="BT10" s="1">
         <v>0</v>
       </c>
-      <c r="BU10" s="2">
+      <c r="BU10" s="1">
         <v>4.6481026999999999</v>
       </c>
-      <c r="BV10" s="2">
+      <c r="BV10" s="1">
         <v>-74.057687899999991</v>
       </c>
       <c r="BW10" t="s">
@@ -4075,7 +3729,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:91" x14ac:dyDescent="0.3">
+    <row r="11">
       <c r="A11" s="1">
         <v>1</v>
       </c>
@@ -4194,7 +3848,7 @@
         <v>253</v>
       </c>
       <c r="AN11" s="1">
-        <v>4.3</v>
+        <v>4.2999999999999998</v>
       </c>
       <c r="AO11" t="s">
         <v>172</v>
@@ -4292,10 +3946,10 @@
       <c r="BT11" s="1">
         <v>0</v>
       </c>
-      <c r="BU11" s="2">
+      <c r="BU11" s="1">
         <v>4.6693340000000001</v>
       </c>
-      <c r="BV11" s="2">
+      <c r="BV11" s="1">
         <v>-74.053410999999997</v>
       </c>
       <c r="BW11" t="s">
@@ -4350,7 +4004,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:91" x14ac:dyDescent="0.3">
+    <row r="12">
       <c r="A12" s="1">
         <v>1</v>
       </c>
@@ -4567,10 +4221,10 @@
       <c r="BT12" s="1">
         <v>0</v>
       </c>
-      <c r="BU12" s="2">
+      <c r="BU12" s="1">
         <v>4.6127433</v>
       </c>
-      <c r="BV12" s="2">
+      <c r="BV12" s="1">
         <v>-74.066767900000002</v>
       </c>
       <c r="BW12" t="s">
@@ -4625,7 +4279,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:91" x14ac:dyDescent="0.3">
+    <row r="13">
       <c r="A13" s="1">
         <v>1</v>
       </c>
@@ -4735,7 +4389,7 @@
         <v>1117</v>
       </c>
       <c r="AK13" s="1">
-        <v>4.7</v>
+        <v>4.7000000000000002</v>
       </c>
       <c r="AL13" s="1">
         <v>1</v>
@@ -4842,10 +4496,10 @@
       <c r="BT13" s="1">
         <v>0</v>
       </c>
-      <c r="BU13" s="2">
+      <c r="BU13" s="1">
         <v>4.6833840000000002</v>
       </c>
-      <c r="BV13" s="2">
+      <c r="BV13" s="1">
         <v>-74.060512199999991</v>
       </c>
       <c r="BW13" t="s">
@@ -4900,7 +4554,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:91" x14ac:dyDescent="0.3">
+    <row r="14">
       <c r="A14" s="1">
         <v>1</v>
       </c>
@@ -5117,10 +4771,10 @@
       <c r="BT14" s="1">
         <v>0</v>
       </c>
-      <c r="BU14" s="2">
+      <c r="BU14" s="1">
         <v>4.6676150999999999</v>
       </c>
-      <c r="BV14" s="2">
+      <c r="BV14" s="1">
         <v>-74.053812199999996</v>
       </c>
       <c r="BW14" t="s">
@@ -5175,7 +4829,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:91" x14ac:dyDescent="0.3">
+    <row r="15">
       <c r="A15" s="1">
         <v>1</v>
       </c>
@@ -5392,10 +5046,10 @@
       <c r="BT15" s="1">
         <v>0</v>
       </c>
-      <c r="BU15" s="2">
+      <c r="BU15" s="1">
         <v>4.6661218999999994</v>
       </c>
-      <c r="BV15" s="2">
+      <c r="BV15" s="1">
         <v>-74.055825599999991</v>
       </c>
       <c r="BW15" t="s">
@@ -5450,7 +5104,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:91" x14ac:dyDescent="0.3">
+    <row r="16">
       <c r="A16" s="1">
         <v>1</v>
       </c>
@@ -5667,10 +5321,10 @@
       <c r="BT16" s="1">
         <v>0</v>
       </c>
-      <c r="BU16" s="2">
+      <c r="BU16" s="1">
         <v>4.6868488000000008</v>
       </c>
-      <c r="BV16" s="2">
+      <c r="BV16" s="1">
         <v>-74.051691300000002</v>
       </c>
       <c r="BW16" t="s">
@@ -5725,7 +5379,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:91" x14ac:dyDescent="0.3">
+    <row r="17">
       <c r="A17" s="1">
         <v>1</v>
       </c>
@@ -5844,7 +5498,7 @@
         <v>220</v>
       </c>
       <c r="AN17" s="1">
-        <v>4.7</v>
+        <v>4.7000000000000002</v>
       </c>
       <c r="AO17" t="s">
         <v>178</v>
@@ -5942,10 +5596,10 @@
       <c r="BT17" s="1">
         <v>0</v>
       </c>
-      <c r="BU17" s="2">
+      <c r="BU17" s="1">
         <v>4.6967935000000001</v>
       </c>
-      <c r="BV17" s="2">
+      <c r="BV17" s="1">
         <v>-74.030623399999996</v>
       </c>
       <c r="BW17" t="s">
@@ -6000,7 +5654,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:91" x14ac:dyDescent="0.3">
+    <row r="18">
       <c r="A18" s="1">
         <v>1</v>
       </c>
@@ -6119,7 +5773,7 @@
         <v>94</v>
       </c>
       <c r="AN18" s="1">
-        <v>4.7</v>
+        <v>4.7000000000000002</v>
       </c>
       <c r="AO18" t="s">
         <v>179</v>
@@ -6217,10 +5871,10 @@
       <c r="BT18" s="1">
         <v>0</v>
       </c>
-      <c r="BU18" s="2">
+      <c r="BU18" s="1">
         <v>4.6459815999999998</v>
       </c>
-      <c r="BV18" s="2">
+      <c r="BV18" s="1">
         <v>-74.059867300000008</v>
       </c>
       <c r="BW18" t="s">
@@ -6275,7 +5929,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:91" x14ac:dyDescent="0.3">
+    <row r="19">
       <c r="A19" s="1">
         <v>1</v>
       </c>
@@ -6394,7 +6048,7 @@
         <v>207</v>
       </c>
       <c r="AN19" s="1">
-        <v>4.2</v>
+        <v>4.2000000000000002</v>
       </c>
       <c r="AO19" t="s">
         <v>180</v>
@@ -6492,10 +6146,10 @@
       <c r="BT19" s="1">
         <v>0</v>
       </c>
-      <c r="BU19" s="2">
+      <c r="BU19" s="1">
         <v>4.6521540999999997</v>
       </c>
-      <c r="BV19" s="2">
+      <c r="BV19" s="1">
         <v>-74.056230099999993</v>
       </c>
       <c r="BW19" t="s">
@@ -6550,7 +6204,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:91" x14ac:dyDescent="0.3">
+    <row r="20">
       <c r="A20" s="1">
         <v>1</v>
       </c>
@@ -6669,7 +6323,7 @@
         <v>48</v>
       </c>
       <c r="AN20" s="1">
-        <v>4.2</v>
+        <v>4.2000000000000002</v>
       </c>
       <c r="AO20" t="s">
         <v>181</v>
@@ -6767,10 +6421,10 @@
       <c r="BT20" s="1">
         <v>0</v>
       </c>
-      <c r="BU20" s="2">
+      <c r="BU20" s="1">
         <v>4.6764162999999996</v>
       </c>
-      <c r="BV20" s="2">
+      <c r="BV20" s="1">
         <v>-74.048835699999998</v>
       </c>
       <c r="BW20" t="s">
@@ -6825,7 +6479,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:91" x14ac:dyDescent="0.3">
+    <row r="21">
       <c r="A21" s="1">
         <v>1</v>
       </c>
@@ -7042,10 +6696,10 @@
       <c r="BT21" s="1">
         <v>0</v>
       </c>
-      <c r="BU21" s="2">
+      <c r="BU21" s="1">
         <v>4.6946344</v>
       </c>
-      <c r="BV21" s="2">
+      <c r="BV21" s="1">
         <v>-74.032175100000018</v>
       </c>
       <c r="BW21" t="s">
@@ -7100,7 +6754,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:91" x14ac:dyDescent="0.3">
+    <row r="22">
       <c r="A22" s="1">
         <v>1</v>
       </c>
@@ -7317,10 +6971,10 @@
       <c r="BT22" s="1">
         <v>0</v>
       </c>
-      <c r="BU22" s="2">
+      <c r="BU22" s="1">
         <v>4.6318294999999994</v>
       </c>
-      <c r="BV22" s="2">
+      <c r="BV22" s="1">
         <v>-74.072424699999999</v>
       </c>
       <c r="BW22" t="s">
@@ -7375,7 +7029,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:91" x14ac:dyDescent="0.3">
+    <row r="23">
       <c r="A23" s="1">
         <v>1</v>
       </c>
@@ -7588,10 +7242,10 @@
       <c r="BT23" s="1">
         <v>0</v>
       </c>
-      <c r="BU23" s="2">
-        <v>4.6560703999999999</v>
-      </c>
-      <c r="BV23" s="2">
+      <c r="BU23" s="1">
+        <v>4.6560704</v>
+      </c>
+      <c r="BV23" s="1">
         <v>-74.054585199999991</v>
       </c>
       <c r="BW23" t="s">
@@ -7646,7 +7300,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:91" x14ac:dyDescent="0.3">
+    <row r="24">
       <c r="A24" s="1">
         <v>1</v>
       </c>
@@ -7863,10 +7517,10 @@
       <c r="BT24" s="1">
         <v>0</v>
       </c>
-      <c r="BU24" s="2">
+      <c r="BU24" s="1">
         <v>4.6944631000000001</v>
       </c>
-      <c r="BV24" s="2">
+      <c r="BV24" s="1">
         <v>-74.032353299999997</v>
       </c>
       <c r="BW24" t="s">
@@ -7921,7 +7575,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:91" x14ac:dyDescent="0.3">
+    <row r="25">
       <c r="A25" s="1">
         <v>1</v>
       </c>
@@ -8040,7 +7694,7 @@
         <v>518</v>
       </c>
       <c r="AN25" s="1">
-        <v>4.3</v>
+        <v>4.2999999999999998</v>
       </c>
       <c r="AO25" t="s">
         <v>186</v>
@@ -8138,10 +7792,10 @@
       <c r="BT25" s="1">
         <v>0</v>
       </c>
-      <c r="BU25" s="2">
+      <c r="BU25" s="1">
         <v>4.6810323999999994</v>
       </c>
-      <c r="BV25" s="2">
+      <c r="BV25" s="1">
         <v>-74.046398499999995</v>
       </c>
       <c r="BW25" t="s">
@@ -8196,7 +7850,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:91" x14ac:dyDescent="0.3">
+    <row r="26">
       <c r="A26" s="1">
         <v>1</v>
       </c>
@@ -8306,7 +7960,7 @@
         <v>171</v>
       </c>
       <c r="AK26" s="1">
-        <v>4.2</v>
+        <v>4.2000000000000002</v>
       </c>
       <c r="AL26" s="1">
         <v>1</v>
@@ -8315,7 +7969,7 @@
         <v>334</v>
       </c>
       <c r="AN26" s="1">
-        <v>4.2</v>
+        <v>4.2000000000000002</v>
       </c>
       <c r="AO26" t="s">
         <v>187</v>
@@ -8413,10 +8067,10 @@
       <c r="BT26" s="1">
         <v>0</v>
       </c>
-      <c r="BU26" s="2">
+      <c r="BU26" s="1">
         <v>4.6963846</v>
       </c>
-      <c r="BV26" s="2">
+      <c r="BV26" s="1">
         <v>-74.044303599999992</v>
       </c>
       <c r="BW26" t="s">
@@ -8471,7 +8125,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:91" x14ac:dyDescent="0.3">
+    <row r="27">
       <c r="A27" s="1">
         <v>1</v>
       </c>
@@ -8590,7 +8244,7 @@
         <v>3</v>
       </c>
       <c r="AN27" s="1">
-        <v>3.3</v>
+        <v>3.2999999999999998</v>
       </c>
       <c r="AO27" t="s">
         <v>188</v>
@@ -8688,10 +8342,10 @@
       <c r="BT27" s="1">
         <v>0</v>
       </c>
-      <c r="BU27" s="2">
+      <c r="BU27" s="1">
         <v>4.6674096</v>
       </c>
-      <c r="BV27" s="2">
+      <c r="BV27" s="1">
         <v>-74.071941100000004</v>
       </c>
       <c r="BW27" t="s">
@@ -8746,7 +8400,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:91" x14ac:dyDescent="0.3">
+    <row r="28">
       <c r="A28" s="1">
         <v>1</v>
       </c>
@@ -8856,7 +8510,7 @@
         <v>126</v>
       </c>
       <c r="AK28" s="1">
-        <v>3.8</v>
+        <v>3.7999999999999998</v>
       </c>
       <c r="AL28" s="1">
         <v>1</v>
@@ -8865,7 +8519,7 @@
         <v>6</v>
       </c>
       <c r="AN28" s="1">
-        <v>3.7</v>
+        <v>3.7000000000000002</v>
       </c>
       <c r="AO28" t="s">
         <v>189</v>
@@ -8963,10 +8617,10 @@
       <c r="BT28" s="1">
         <v>0</v>
       </c>
-      <c r="BU28" s="2">
-        <v>4.6130630999999997</v>
-      </c>
-      <c r="BV28" s="2">
+      <c r="BU28" s="1">
+        <v>4.6130630999999998</v>
+      </c>
+      <c r="BV28" s="1">
         <v>-74.06663069999999</v>
       </c>
       <c r="BW28" t="s">
@@ -9021,7 +8675,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:91" x14ac:dyDescent="0.3">
+    <row r="29">
       <c r="A29" s="1">
         <v>1</v>
       </c>
@@ -9234,10 +8888,10 @@
       <c r="BT29" s="1">
         <v>0</v>
       </c>
-      <c r="BU29" s="2">
+      <c r="BU29" s="1">
         <v>4.6521447</v>
       </c>
-      <c r="BV29" s="2">
+      <c r="BV29" s="1">
         <v>-74.055869399999992</v>
       </c>
       <c r="BW29" t="s">
@@ -9292,7 +8946,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:91" x14ac:dyDescent="0.3">
+    <row r="30">
       <c r="A30" s="1">
         <v>1</v>
       </c>
@@ -9402,7 +9056,7 @@
         <v>87</v>
       </c>
       <c r="AK30" s="1">
-        <v>4.7</v>
+        <v>4.7000000000000002</v>
       </c>
       <c r="AL30" s="1">
         <v>1</v>
@@ -9411,7 +9065,7 @@
         <v>24</v>
       </c>
       <c r="AN30" s="1">
-        <v>4.7</v>
+        <v>4.7000000000000002</v>
       </c>
       <c r="AO30" t="s">
         <v>190</v>
@@ -9509,10 +9163,10 @@
       <c r="BT30" s="1">
         <v>0</v>
       </c>
-      <c r="BU30" s="2">
+      <c r="BU30" s="1">
         <v>4.6742881000000001</v>
       </c>
-      <c r="BV30" s="2">
+      <c r="BV30" s="1">
         <v>-74.048050799999999</v>
       </c>
       <c r="BW30" t="s">
@@ -9567,7 +9221,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:91" x14ac:dyDescent="0.3">
+    <row r="31">
       <c r="A31" s="1">
         <v>1</v>
       </c>
@@ -9677,7 +9331,7 @@
         <v>85</v>
       </c>
       <c r="AK31" s="1">
-        <v>3.9</v>
+        <v>3.8999999999999999</v>
       </c>
       <c r="AL31" s="1">
         <v>0</v>
@@ -9780,10 +9434,10 @@
       <c r="BT31" s="1">
         <v>0</v>
       </c>
-      <c r="BU31" s="2">
+      <c r="BU31" s="1">
         <v>4.6009235999999998</v>
       </c>
-      <c r="BV31" s="2">
+      <c r="BV31" s="1">
         <v>-74.07176849999999</v>
       </c>
       <c r="BW31" t="s">
@@ -9838,7 +9492,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:91" x14ac:dyDescent="0.3">
+    <row r="32">
       <c r="A32" s="1">
         <v>1</v>
       </c>
@@ -10051,10 +9705,10 @@
       <c r="BT32" s="1">
         <v>0</v>
       </c>
-      <c r="BU32" s="2">
+      <c r="BU32" s="1">
         <v>4.6645292999999999</v>
       </c>
-      <c r="BV32" s="2">
+      <c r="BV32" s="1">
         <v>-74.063854599999999</v>
       </c>
       <c r="BW32" t="s">
@@ -10109,7 +9763,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:91" x14ac:dyDescent="0.3">
+    <row r="33">
       <c r="A33" s="1">
         <v>1</v>
       </c>
@@ -10183,7 +9837,7 @@
         <v>3.2999999523162842</v>
       </c>
       <c r="Y33" s="1">
-        <v>4.4000000953674316</v>
+        <v>4.4000000953674317</v>
       </c>
       <c r="Z33" s="1">
         <v>2.2000000476837158</v>
@@ -10326,10 +9980,10 @@
       <c r="BT33" s="1">
         <v>0</v>
       </c>
-      <c r="BU33" s="2">
+      <c r="BU33" s="1">
         <v>4.6509020999999997</v>
       </c>
-      <c r="BV33" s="2">
+      <c r="BV33" s="1">
         <v>-74.057391199999998</v>
       </c>
       <c r="BW33" t="s">
@@ -10384,7 +10038,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:91" x14ac:dyDescent="0.3">
+    <row r="34">
       <c r="A34" s="1">
         <v>1</v>
       </c>
@@ -10599,10 +10253,10 @@
       <c r="BT34" s="1">
         <v>0</v>
       </c>
-      <c r="BU34" s="2">
-        <v>4.5965129999999998</v>
-      </c>
-      <c r="BV34" s="2">
+      <c r="BU34" s="1">
+        <v>4.5965129999999999</v>
+      </c>
+      <c r="BV34" s="1">
         <v>-74.069208899999992</v>
       </c>
       <c r="BW34" t="s">
@@ -10657,7 +10311,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:91" x14ac:dyDescent="0.3">
+    <row r="35">
       <c r="A35" s="1">
         <v>1</v>
       </c>
@@ -10767,7 +10421,7 @@
         <v>11</v>
       </c>
       <c r="AK35" s="1">
-        <v>4.7</v>
+        <v>4.7000000000000002</v>
       </c>
       <c r="AL35" s="1">
         <v>0</v>
@@ -10870,10 +10524,10 @@
       <c r="BT35" s="1">
         <v>0</v>
       </c>
-      <c r="BU35" s="2">
+      <c r="BU35" s="1">
         <v>4.6574445999999998</v>
       </c>
-      <c r="BV35" s="2">
+      <c r="BV35" s="1">
         <v>-74.05652529999999</v>
       </c>
       <c r="BW35" t="s">
@@ -10928,7 +10582,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:91" x14ac:dyDescent="0.3">
+    <row r="36">
       <c r="A36" s="1">
         <v>1</v>
       </c>
@@ -11047,7 +10701,7 @@
         <v>1231</v>
       </c>
       <c r="AN36" s="1">
-        <v>4.3</v>
+        <v>4.2999999999999998</v>
       </c>
       <c r="AO36" t="s">
         <v>192</v>
@@ -11145,10 +10799,10 @@
       <c r="BT36" s="1">
         <v>0</v>
       </c>
-      <c r="BU36" s="2">
+      <c r="BU36" s="1">
         <v>4.6859608000000001</v>
       </c>
-      <c r="BV36" s="2">
+      <c r="BV36" s="1">
         <v>-74.054435400000003</v>
       </c>
       <c r="BW36" t="s">
@@ -11204,6 +10858,5 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>